<commit_message>
Ship Client Revision Batch 2: copy honesty, forms, sample, and legal gates.
Replace draft WhatsApp/acquisition/probate language, lock sample subtotals and MasterFormat naming, add short contact + plan-room + Blob upload path, soften licensing, and gate company identity until the owner supplies it.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/public/samples/sample-estimate.xlsx
+++ b/frontend/public/samples/sample-estimate.xlsx
@@ -128,7 +128,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>06 Wood &amp; Plastics</t>
+          <t>06 Wood, Plastics, and Composites</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -145,7 +145,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07 Thermal &amp; Moisture</t>
+          <t>07 Thermal &amp; Moisture Protection</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -179,7 +179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sample total</t>
+          <t>Subtotal, divisions shown</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -215,7 +215,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Illustrative sample. Div 03 totals are live formulas from the Div 03 sheet.</t>
+          <t>Illustrative sample — divisions shown only. Div 08 Openings omitted. Div 03 totals are live formulas from the Div 03 sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>